<commit_message>
Fix slot win reset and result format
</commit_message>
<xml_diff>
--- a/ExcelTable/Config.xlsx
+++ b/ExcelTable/Config.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SlotMachineConfig" sheetId="1" r:id="Rfdddd6bc41664875"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CurrencyConfig" sheetId="2" r:id="R1dceaa6770774a27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SlotMachineConfig" sheetId="1" r:id="Rba9b8cd074644948"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CurrencyConfig" sheetId="2" r:id="R0fb9cedc4754439d"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>